<commit_message>
R├®paration de postion tr├®sor temporairement
</commit_message>
<xml_diff>
--- a/Calcul_coup_possible.xlsx
+++ b/Calcul_coup_possible.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elkat\Documents\Github\Gitlabsu\Jeu_labyrinthe\jeu_labyrinthe_yek\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C948BE-ED63-4F14-82B5-30AE0EBC80A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ECF764D-B0ED-4DB0-B605-B87F92236CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="14400" windowHeight="15600" xr2:uid="{2757F9AD-9C7C-4B0C-9B04-EBC4D55791A6}"/>
+    <workbookView xWindow="14400" yWindow="600" windowWidth="14400" windowHeight="15600" xr2:uid="{2757F9AD-9C7C-4B0C-9B04-EBC4D55791A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -487,7 +487,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -495,7 +495,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -512,7 +512,7 @@
       </c>
       <c r="B5" s="4">
         <f>INT(B2/2)</f>
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -521,7 +521,7 @@
       </c>
       <c r="B6" s="4">
         <f>INT(B3/2)</f>
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -533,7 +533,7 @@
       </c>
       <c r="B8" s="4">
         <f>B5*2</f>
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -542,7 +542,7 @@
       </c>
       <c r="B9" s="4">
         <f>B6*2</f>
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -551,7 +551,7 @@
       </c>
       <c r="B10" s="4">
         <f>B8+B9</f>
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -560,7 +560,7 @@
       </c>
       <c r="B11" s="4">
         <f>B10*B4</f>
-        <v>152</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>